<commit_message>
Dien san phuong an Microsoft 365 Copilot: pham vi, chan doan, workflow moi, dashboard 7 chi so
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dashboard/dashboard_hanh_dong_v2.xlsx
+++ b/dashboard/dashboard_hanh_dong_v2.xlsx
@@ -505,9 +505,9 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Nhóm: B2    |    Phạm vi: &lt;1 sản phẩm AI · 1 nhóm người dùng · 2–4 quy trình&gt;</t>
+      <c r="A2" s="9" t="inlineStr">
+        <is>
+          <t>Nhóm: B2    |    Phạm vi: Microsoft 365 Copilot (đã cấp license toàn phòng) · nhân viên khối văn phòng · 3 quy trình: soạn văn bản, tóm tắt cuộc họp, tra cứu tài liệu trên SharePoint</t>
         </is>
       </c>
     </row>
@@ -565,190 +565,334 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+    <row r="6" ht="62" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>1. Sử dụng</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Workflow</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Tỷ lệ ca soạn văn bản đi qua bước dùng Copilot theo quy trình chuẩn</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Đo tuần 1: đếm trên mẫu 30 ca soạn văn bản của phòng</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>≥ 60% sau 60 ngày (chốt lại sau khi có baseline)</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="inlineStr">
+        <is>
+          <t>Log quy trình của phòng + báo cáo sử dụng Microsoft 365 admin center</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>Trưởng nhóm văn phòng</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>Tìm điểm vướng: phỏng vấn 3 người đã bỏ dùng, xác định bước nào gây bỏ cuộc</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>Đếm theo quy trình, không đếm số lần đăng nhập</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="62" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>2. Hành vi</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Workflow</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Tỷ lệ người dùng mở tài liệu nguồn để kiểm chứng trước khi dùng kết quả</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Đo tuần 1: quan sát tại chỗ 10 ca + khảo sát ngắn</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>≥ 80% sau 60 ngày</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Quan sát mẫu hàng tuần + khảo sát 5 câu</t>
+        </is>
+      </c>
+      <c r="G7" s="7" t="inlineStr">
+        <is>
+          <t>Trưởng nhóm văn phòng</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Bổ sung hướng dẫn kiểm chứng ngay trong quy trình, không mở lớp đào tạo rời</t>
+        </is>
+      </c>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>Đo thay đổi cách làm việc, không đo thái độ</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="62" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>3. Năng suất</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Workflow</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Thời gian trung bình hoàn thành một văn bản chuẩn (phút)</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Đo hiện trạng: bấm giờ mẫu 20 ca trước khi đổi quy trình</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Giảm ≥ 25% so với baseline</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Log tác vụ / hệ thống giao việc, không dùng số tự khai</t>
+        </is>
+      </c>
+      <c r="G8" s="7" t="inlineStr">
+        <is>
+          <t>Chủ quy trình soạn văn bản</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>Xem lại cách làm: kiểm tra bước nào bị thêm thời gian vì phải kiểm chứng thủ công</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>Không dùng chỉ số thời gian tiết kiệm do người dùng tự khai</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="62" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>4. Chất lượng &amp; tin cậy</t>
         </is>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>VÍ DỤ: Tỷ lệ câu trả lời có nguồn kiểm chứng</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>Đo mẫu 30 câu tuần 1 (vd 40%)</t>
-        </is>
-      </c>
-      <c r="E6" s="5" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Tỷ lệ câu trả lời truy được về tài liệu nguồn có ngày cập nhật</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Đo mẫu tuần 1: 30 câu hỏi thật của nhân viên</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>≥ 90% sau 60 ngày</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Kiểm tra mẫu hàng tuần (QA)</t>
-        </is>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Kiểm tra mẫu 30 câu/tuần do QA chấm</t>
+        </is>
+      </c>
+      <c r="G9" s="7" t="inlineStr">
         <is>
           <t>Phụ trách QA</t>
         </is>
       </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>Tăng kiểm soát: bật bắt buộc trích nguồn, rà lại nguồn thiếu</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>Minh hoạ theo ví dụ §3.3 — xoá dòng này</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>1. Sử dụng</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Tăng kiểm soát: thu hẹp phạm vi tài liệu về kho đã có owner, bắt buộc hiện nguồn</t>
+        </is>
+      </c>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>PRODUCT METRIC bắt buộc — gắn trực tiếp với nguyên nhân gốc độ tin cậy</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="62" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>4. Chất lượng &amp; tin cậy</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Workflow</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>Mức dùng theo quy trình</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
-      <c r="F7" s="7" t="inlineStr"/>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr"/>
-      <c r="I7" s="7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>2. Hành vi</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>Workflow</t>
-        </is>
-      </c>
-      <c r="C8" s="7" t="inlineStr">
-        <is>
-          <t>Cách làm việc có thay đổi không</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr"/>
-      <c r="E8" s="7" t="inlineStr"/>
-      <c r="F8" s="7" t="inlineStr"/>
-      <c r="G8" s="7" t="inlineStr"/>
-      <c r="H8" s="7" t="inlineStr"/>
-      <c r="I8" s="7" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>3. Năng suất</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Workflow</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>Thời gian / năng suất (từ log tác vụ)</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr"/>
-      <c r="E9" s="7" t="inlineStr"/>
-      <c r="F9" s="7" t="inlineStr"/>
-      <c r="G9" s="7" t="inlineStr"/>
-      <c r="H9" s="7" t="inlineStr"/>
-      <c r="I9" s="7" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>4. Chất lượng &amp; tin cậy</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>Tỷ lệ bản nháp dùng được mà không phải viết lại từ đầu</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Đo mẫu tuần 1: 20 bản nháp</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>≥ 70% sau 60 ngày</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>Đánh giá mẫu bởi người duyệt văn bản</t>
+        </is>
+      </c>
+      <c r="G10" s="7" t="inlineStr">
+        <is>
+          <t>Người duyệt văn bản</t>
+        </is>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>Rà soát lại mẫu nhắc và phạm vi tài liệu; nếu không cải thiện thì thu hẹp use case</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="inlineStr">
+        <is>
+          <t>Đo chất lượng đầu ra, không đo số lượng</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="62" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>5. Giá trị</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="C10" s="7" t="inlineStr">
-        <is>
-          <t>Chất lượng / tin cậy (vd tỷ lệ có nguồn, tỷ lệ không làm lại)</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr"/>
-      <c r="E10" s="7" t="inlineStr"/>
-      <c r="F10" s="7" t="inlineStr"/>
-      <c r="G10" s="7" t="inlineStr"/>
-      <c r="H10" s="7" t="inlineStr"/>
-      <c r="I10" s="7" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>5. Giá trị</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Thời gian chờ trung bình để hoàn thành một yêu cầu văn bản nội bộ (từ lúc nhận đến lúc phát hành)</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Số hiện tại lấy từ hệ thống giao việc 3 tháng gần nhất</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>Giảm ≥ 20% sau 90 ngày</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Hệ thống giao việc / quản lý công việc của phòng</t>
+        </is>
+      </c>
+      <c r="G11" s="7" t="inlineStr">
+        <is>
+          <t>Chủ nghiệp vụ (trưởng phòng)</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>Điều chỉnh hoặc dừng: sau 90 ngày không cải thiện thì trả license và đóng pilot</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr">
+        <is>
+          <t>Kết quả nghiệp vụ, không phải chỉ số sử dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="62" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Rủi ro / bàn giao</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>Kết quả nghiệp vụ</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr"/>
-      <c r="E11" s="7" t="inlineStr"/>
-      <c r="F11" s="7" t="inlineStr"/>
-      <c r="G11" s="7" t="inlineStr"/>
-      <c r="H11" s="7" t="inlineStr"/>
-      <c r="I11" s="7" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>Rủi ro / bàn giao</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="C12" s="7" t="inlineStr">
-        <is>
-          <t>Rủi ro / bàn giao (lỗi, chuyển người)</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr"/>
-      <c r="E12" s="7" t="inlineStr"/>
-      <c r="F12" s="7" t="inlineStr"/>
-      <c r="G12" s="7" t="inlineStr"/>
-      <c r="H12" s="7" t="inlineStr"/>
-      <c r="I12" s="7" t="inlineStr"/>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>Số ca Copilot đưa thông tin sai hoặc trích sai nguồn được báo cáo</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>Ghi hiện trạng từ tuần 1 khi bật nút báo lỗi</t>
+        </is>
+      </c>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>Ngưỡng nhóm: ≤ 2 ca/tuần, không có ca gây hậu quả ra ngoài</t>
+        </is>
+      </c>
+      <c r="F12" s="7" t="inlineStr">
+        <is>
+          <t>Log lỗi từ nút báo lỗi đặt trong quy trình</t>
+        </is>
+      </c>
+      <c r="G12" s="7" t="inlineStr">
+        <is>
+          <t>Phụ trách AI của phòng</t>
+        </is>
+      </c>
+      <c r="H12" s="7" t="inlineStr">
+        <is>
+          <t>Bổ sung xử lý: tắt phạm vi tài liệu chưa có owner, thêm bước người duyệt bắt buộc</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr">
+        <is>
+          <t>Có cơ chế báo lỗi thì mới học được từ lỗi</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Them sheet Workflow AS-IS / TO-BE vao dashboard v1 va v2
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dashboard/dashboard_hanh_dong_v2.xlsx
+++ b/dashboard/dashboard_hanh_dong_v2.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Huong_dan" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workflow_ASIS_TOBE" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Huong_dan" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,8 +49,13 @@
       <i val="1"/>
       <color rgb="00777777"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -66,8 +72,18 @@
         <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -89,11 +105,55 @@
         <color rgb="00999999"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="00999999"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00999999"/>
+      </right>
+      <top style="thin">
+        <color rgb="00999999"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00999999"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -118,6 +178,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -908,6 +981,305 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Workflow AS-IS / TO-BE — Microsoft 365 Copilot, khối văn phòng</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Ô nền vàng là chỗ nhóm cần sửa theo tình huống thật. Nguyên tắc chấm: TO-BE phải khác AS-IS ở cách chia việc và trách nhiệm, không phải chỉ chèn thêm một bước hỏi AI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>1. Ba quy trình trong phạm vi</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Quy trình</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>AS-IS — cách làm hiện tại</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>TO-BE — cách làm mới</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Thay đổi thật sự nằm ở đâu</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="108" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Soạn văn bản</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>1. Nhận yêu cầu
+2. Tự mở thư mục tìm văn bản mẫu cũ
+3. Soạn tay từ đầu hoặc copy bản cũ
+4. Gửi người duyệt</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>1. Nhận yêu cầu
+2. Hỏi Copilot theo mẫu nhắc chuẩn của phòng
+3. Mở tài liệu nguồn Copilot trích, kiểm ngày cập nhật
+4. Soạn và chịu trách nhiệm nội dung cuối
+5. Gửi người duyệt, hoặc bấm báo lỗi và quay về cách cũ</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Thêm bước kiểm chứng nguồn bắt buộc trước khi dùng, và có đường lui rõ ràng khi không truy được nguồn</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="108" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Tóm tắt cuộc họp</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>1. Người ghi biên bản tự nghe lại và gõ
+2. Gửi bản tóm tắt qua email
+3. Không ai đối chiếu lại với bản ghi</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>1. Copilot tạo bản tóm tắt kèm mốc thời gian trong bản ghi
+2. Chủ trì cuộc họp đối chiếu các mục quyết định và việc được giao
+3. Chủ trì xác nhận rồi mới phát hành
+4. Sai thì sửa và bấm báo lỗi</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Chuyển việc gõ sang AI, nhưng đưa trách nhiệm xác nhận về đúng người chủ trì thay vì không ai kiểm</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="108" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Tra cứu tài liệu SharePoint</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>1. Tự đoán tài liệu nằm ở site nào
+2. Mở nhiều thư mục, hỏi đồng nghiệp
+3. Dùng bản tìm được, khó biết có phải bản mới nhất</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>1. Hỏi Copilot, chỉ trên các kho đã có người phụ trách
+2. Copilot trả về câu trả lời kèm liên kết nguồn và ngày cập nhật
+3. Người dùng mở nguồn kiểm chứng
+4. Không có nguồn hoặc nguồn quá hạn thì quay về cách cũ và báo lỗi</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Thu hẹp phạm vi về kho có owner, và biến ngày cập nhật thành điều kiện để được dùng kết quả</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>2. Ba thay đổi bắt buộc</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Thay đổi</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Nội dung</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="62" customHeight="1">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Nguồn kiểm chứng</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Chỉ bật Copilot trên kho SharePoint đã có người phụ trách nội dung và lịch cập nhật. Mọi câu trả lời phải kèm liên kết tài liệu nguồn và ngày cập nhật. Không có nguồn thì không dùng.</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="n"/>
+      <c r="D12" s="15" t="n"/>
+    </row>
+    <row r="13" ht="62" customHeight="1">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>Người chịu trách nhiệm</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Người soạn văn bản chịu trách nhiệm kết quả cuối và phải mở tài liệu nguồn kiểm chứng trước khi gửi. Người duyệt văn bản giữ quyền phê duyệt. Với biên bản họp, người chủ trì là người xác nhận.</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="n"/>
+      <c r="D13" s="15" t="n"/>
+    </row>
+    <row r="14" ht="62" customHeight="1">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Cách xử lý khi AI không chắc</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Không truy được nguồn hoặc nguồn quá hạn cập nhật thì chuyển về cách làm cũ và bấm nút báo lỗi. Log lỗi được rà hàng tuần, là đầu vào để thu hẹp hoặc mở rộng phạm vi tài liệu.</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="n"/>
+      <c r="D14" s="15" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>3. Phân chia việc người – AI (Mollick)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>Vùng</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Nội dung trong ba quy trình này</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="50" customHeight="1">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>Người giữ quyền</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
+        <is>
+          <t>Phê duyệt văn bản phát hành, xác nhận biên bản họp, xử lý ngoại lệ, chịu trách nhiệm nội dung cuối</t>
+        </is>
+      </c>
+      <c r="C18" s="14" t="n"/>
+      <c r="D18" s="15" t="n"/>
+    </row>
+    <row r="19" ht="50" customHeight="1">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>AI hỗ trợ, người kiểm</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>Copilot dựng bản nháp, tóm tắt cuộc họp, tìm và trích tài liệu. Người dùng kiểm chứng nguồn trước khi dùng. Cả ba quy trình đều nằm ở vùng này.</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="n"/>
+      <c r="D19" s="15" t="n"/>
+    </row>
+    <row r="20" ht="50" customHeight="1">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>AI tự động</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>Không có phần nào trong ba quy trình này được tự động hoàn toàn, vì văn bản phát hành có rủi ro và chưa có tiêu chí kiểm tra tự động.</t>
+        </is>
+      </c>
+      <c r="C20" s="14" t="n"/>
+      <c r="D20" s="15" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>4. Kiến trúc tin cậy</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>Nguồn → Trích nguồn → QA mẫu → Chuyển người → Phản hồi</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="46" customHeight="1">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>Nguồn: chỉ kho có người phụ trách và lịch cập nhật. Trích nguồn: câu trả lời kèm liên kết và ngày cập nhật. QA mẫu: 30 câu mỗi tuần do QA chấm. Chuyển người: người soạn và người duyệt chịu trách nhiệm cuối. Phản hồi: nút báo lỗi, log rà hàng tuần.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="8">
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="B14:D14"/>
+    <mergeCell ref="B18:D18"/>
+    <mergeCell ref="B13:D13"/>
+    <mergeCell ref="A24:D24"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="B12:D12"/>
+    <mergeCell ref="B20:D20"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Dien baseline/target gia dinh co neo, hoan thien memo va quyet dinh; v1 khac v2 hai diem
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dashboard/dashboard_hanh_dong_v2.xlsx
+++ b/dashboard/dashboard_hanh_dong_v2.xlsx
@@ -587,7 +587,7 @@
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Hướng dẫn: điền các ô nền vàng. Mỗi chỉ số phải đủ 5 cột: Mốc đầu · Mục tiêu · Nguồn dữ liệu · Phụ trách · Khi chỉ số xấu. Chỉ đặt mục tiêu cho chỉ số nhóm lấy được số liệu thật. Dòng 'VÍ DỤ' chỉ minh hoạ cách điền — xoá trước khi nộp.</t>
+          <t>Hướng dẫn: ô nền vàng là ô nhóm điền. Các số đánh dấu (giả định) là số nháp để minh hoạ logic ra quyết định, phải thay bằng số đo thật trước khi dùng cho quyết định thật; căn cứ của từng giả định ghi ở cột Ghi chú.</t>
         </is>
       </c>
     </row>
@@ -656,12 +656,12 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Đo tuần 1: đếm trên mẫu 30 ca soạn văn bản của phòng</t>
+          <t>25% (giả định, mẫu 30 ca tuần 1)</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>≥ 60% sau 60 ngày (chốt lại sau khi có baseline)</t>
+          <t>≥ 60% sau 60 ngày</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="I6" s="7" t="inlineStr">
         <is>
-          <t>Đếm theo quy trình, không đếm số lần đăng nhập</t>
+          <t>Baseline neo theo GDS: 25% dùng Copilot hằng ngày trong Word. Target neo theo DBT: 64% người dùng hoạt động theo tuần.</t>
         </is>
       </c>
     </row>
@@ -703,7 +703,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Đo tuần 1: quan sát tại chỗ 10 ca + khảo sát ngắn</t>
+          <t>30% (giả định, quan sát 10 ca)</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -750,12 +750,12 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Đo hiện trạng: bấm giờ mẫu 20 ca trước khi đổi quy trình</t>
+          <t>48 phút (giả định, bấm giờ mẫu 20 ca)</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>Giảm ≥ 25% so với baseline</t>
+          <t>≤ 36 phút, giảm 25%</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
@@ -775,7 +775,7 @@
       </c>
       <c r="I8" s="7" t="inlineStr">
         <is>
-          <t>Không dùng chỉ số thời gian tiết kiệm do người dùng tự khai</t>
+          <t>DBT cảnh báo thời gian tự khai lệch với thời gian đo thật, nên chỉ lấy từ log</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>Đo mẫu tuần 1: 30 câu hỏi thật của nhân viên</t>
+          <t>45% (giả định, mẫu 30 câu hỏi thật)</t>
         </is>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -844,7 +844,7 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Đo mẫu tuần 1: 20 bản nháp</t>
+          <t>40% (giả định, mẫu 20 bản nháp)</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -854,7 +854,7 @@
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Đánh giá mẫu bởi người duyệt văn bản</t>
+          <t>Đánh giá mẫu bởi người duyệt văn bản, thang điểm 1–5, đạt từ 4 trở lên</t>
         </is>
       </c>
       <c r="G10" s="7" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
-          <t>Đo chất lượng đầu ra, không đo số lượng</t>
+          <t>Thêm ở v2, thay cho chỉ số đếm số câu hỏi. DBT chấm chất lượng trên thang 1–5, nhóm dùng lại cách này.</t>
         </is>
       </c>
     </row>
@@ -891,12 +891,12 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Số hiện tại lấy từ hệ thống giao việc 3 tháng gần nhất</t>
+          <t>3,5 ngày làm việc (giả định, 3 tháng gần nhất)</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>Giảm ≥ 20% sau 90 ngày</t>
+          <t>≤ 2,8 ngày, giảm 20% sau 90 ngày</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="I11" s="7" t="inlineStr">
         <is>
-          <t>Kết quả nghiệp vụ, không phải chỉ số sử dụng</t>
+          <t>Kết quả nghiệp vụ, là chỉ số quyết định ở cổng 90 ngày</t>
         </is>
       </c>
     </row>
@@ -938,12 +938,12 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Ghi hiện trạng từ tuần 1 khi bật nút báo lỗi</t>
+          <t>Chưa đo được: chưa có nút báo lỗi nên hiện ghi nhận 0 ca, không dùng để so sánh</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>Ngưỡng nhóm: ≤ 2 ca/tuần, không có ca gây hậu quả ra ngoài</t>
+          <t>Ngưỡng nhóm: ≤ 2 ca/tuần, không có ca lọt ra ngoài phòng</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="I12" s="7" t="inlineStr">
         <is>
-          <t>Có cơ chế báo lỗi thì mới học được từ lỗi</t>
+          <t>Thêm ở v2. DBT ghi nhận có hiện tượng bịa thông tin, nên bắt buộc phải có kênh ghi nhận.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bo ghi chu nhap, them lo trinh 30-60-90 vao README, tro toi sheet AS-IS/TO-BE, sua chu giai v1/v2
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dashboard/dashboard_hanh_dong_v2.xlsx
+++ b/dashboard/dashboard_hanh_dong_v2.xlsx
@@ -1280,7 +1280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -1296,7 +1296,7 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Ô nền vàng = ô nhóm cần điền.</t>
+          <t>Ô nền vàng là ô dữ liệu nhóm điền. Các số ghi kèm chữ (giả định) là số nháp có neo vào nguồn công khai, căn cứ neo ghi ở cột Ghi chú của sheet Dashboard; phải thay bằng số đo thật trước khi dùng cho quyết định thật.</t>
         </is>
       </c>
     </row>
@@ -1373,6 +1373,20 @@
       <c r="A14" s="9" t="inlineStr">
         <is>
           <t>Đủ mạnh để quyết: thời gian xử lý từ log, tỷ lệ hoàn thành không cần QA làm lại, tỷ lệ câu trả lời có nguồn, kết quả nghiệp vụ theo workflow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Bản này là gì</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="9" t="inlineStr">
+        <is>
+          <t>Bản v2 — sau kiểm tra chéo. Có 7 chỉ số. Hai thay đổi so với v1: bỏ chỉ số đếm số câu hỏi và thay bằng 'Tỷ lệ bản nháp dùng được mà không phải viết lại'; thêm dòng rủi ro / bàn giao 'Số ca đưa thông tin sai hoặc trích sai nguồn' kèm owner và hành động.</t>
         </is>
       </c>
     </row>

</xml_diff>